<commit_message>
add save window and multi panel saving
</commit_message>
<xml_diff>
--- a/app/database/database_test_1.xlsx
+++ b/app/database/database_test_1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10311"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/u0065634/Documents/Software_projects/msi-quant/app/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEA66BFB-2408-6245-AA7E-C9496F6D0D2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAF3A6AA-87F8-514C-842C-72BF6B630C65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3340" yWindow="2000" windowWidth="30240" windowHeight="17780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -137,7 +137,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -155,6 +155,12 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -865,6 +871,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>